<commit_message>
mlflow code with version1
</commit_message>
<xml_diff>
--- a/Data/shuffled_sat_items.xlsx
+++ b/Data/shuffled_sat_items.xlsx
@@ -413,71 +413,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>question_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>question_type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>source_text</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>sentence</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>editable_portion</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>option_a</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>option_b</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>option_c</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>option_d</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>correct_answer</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>explanation</t>
         </is>
@@ -486,3169 +491,3075 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Expression of Ideas</t>
+          <t>4f78c32d-71b7-4abf-b9d3-f48828300f04</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Transitions</t>
+          <t>Craft and Structure</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Words in Context</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Many renewable energy projects require significant initial investment. However, their long-term benefits often outweigh the upfront costs.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Many renewable energy projects require significant initial investment. However, their long-term benefits often outweigh the upfront costs.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>However</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Which choice best connects the ideas in the text?</t>
-        </is>
-      </c>
+          <t>When studying the migration of birds, scientists observe both predictable and unpredictable patterns. Some species follow a consistent route each year, demonstrating a reliable journey. However, other species display erratic movements, changing their paths depending on weather and food availability. The word 'erratic' is used here to describe behavior that is irregular, not steady like the predictable routes of other birds.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>For example</t>
+          <t>In the passage, what does the word 'erratic' most nearly mean?</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Consequently</t>
+          <t>Irregular</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>However</t>
+          <t>Consistent</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Similarly</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Predictable</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The transition 'However' correctly establishes a contrast between the initial costs and the long-term benefits of renewable energy projects.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>The passage contrasts the predictable routes of some bird species with the 'erratic movements' of others, which change based on weather and food availability. This context indicates that 'erratic' means irregular.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Expression of Ideas</t>
+          <t>ecca2a38-b04e-4376-a4ad-e44d58e05ebf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Transitions</t>
+          <t>Craft and Structure</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Words in Context</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>The researchers expected the experimental treatment to improve memory performance; ___, the results showed no significant difference between the treatment and control groups.</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The researchers expected the experimental treatment to improve memory performance; ___, the results showed no significant difference between the treatment and control groups.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>___</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Which choice best connects the ideas in the text?</t>
-        </is>
-      </c>
+          <t>In the study of ecosystems, the term 'resilience' refers to an environment’s ability to recover from disturbances, such as fires or floods. While some scientists interpret resilience as mere persistence, others argue that true resilience entails adaptation—an ecosystem not only returns to its previous state, but evolves in response to challenges. Thus, the meaning of 'resilience' in ecological research is not static; rather, it is continually redefined as our understanding of environmental dynamics expands.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>meanwhile</t>
+          <t>In the passage, what does the word 'resilience' most nearly mean?</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>therefore</t>
+          <t>The ability to recover and adapt</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>however</t>
+          <t>Simple persistence</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>furthermore</t>
+          <t>A static condition</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Immediate recovery</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>The sentence presents an expectation that is contradicted by the actual results of the experiment. The logical relationship is one of contrast, making 'however' the correct transition to use.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>The passage explains that while some interpret 'resilience' as mere persistence, others argue it involves adaptation, indicating it means the ability to recover and adapt.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Expression of Ideas</t>
+          <t>8d288abf-78b4-4449-ae2a-1ab1971afbff</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Transitions</t>
+          <t>Craft and Structure</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Words in Context</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The invention of the printing press greatly increased access to books. However, literacy rates remained low for many years afterward.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The invention of the printing press greatly increased access to books. However, literacy rates remained low for many years afterward.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>However,</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Which choice best connects the ideas in the text?</t>
-        </is>
-      </c>
+          <t>While the term 'paradigm' is frequently invoked to denote a prevailing framework of thought, its application in scientific discourse often assumes a more circumscribed meaning. Thomas Kuhn's seminal work, for example, differentiates between a paradigm as a comprehensive model guiding research and the mere accumulation of scientific facts. This distinction underscores the pivotal role of paradigms in not only shaping inquiry but also in delimiting the boundaries of acceptable interpretation. Thus, to conflate paradigms with simple scientific consensus is to overlook their function as both catalysts for innovation and, paradoxically, as constraints on intellectual exploration.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>For example,</t>
+          <t>In the context of the passage, what is the meaning of the word 'conflate'?</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>However,</t>
+          <t>support with evidence</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Consequently,</t>
+          <t>combine two distinct concepts into one</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Similarly,</t>
+          <t>analyze thoroughly</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>dismiss as unimportant</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>The sentence presents a contrast between the increased access to books and the persistent low literacy rates, making 'However,' the most appropriate transition to express this contrast.</t>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>In the passage, 'conflate' is used to describe the mistake of incorrectly merging the idea of paradigms with scientific consensus, suggesting that it means to combine two distinct concepts into one.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>4b2090c8-297c-4c77-86ae-91378ee78132</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Words in Context</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Text Structure</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>At first, the scientist was reluctant to share her findings with the public. She worried that people might misunderstand her results or question her methods. However, after careful consideration, she decided to present her research at a conference. The positive feedback she received boosted her confidence, leading her to publish her work in a scientific journal, where it sparked a lively discussion among experts. Her confidence grew as more colleagues expressed interest in her discoveries, giving her the courage to continue her research.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Many historians believe that the invention of the printing press was the most important event in the spread of knowledge during the Renaissance. They argue that printed books allowed ideas to reach more people than ever before, making education more accessible. However, some scholars contend that other factors, such as the rise of universities and improved transportation, played equally significant roles in sharing information. Nevertheless, most agree that the printing press changed the way people learned and communicated in Europe.</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>As used in the passage, what does the word 'reluctant' most nearly mean?</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>eager</t>
+          <t>How does the passage structure the discussion of the printing press's role in the spread of knowledge during the Renaissance?</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>confident</t>
+          <t>It provides a chronological account of the development of the printing press.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>unwilling</t>
+          <t>It critiques the effectiveness of the printing press in comparison to modern technology.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>hesitant</t>
+          <t>It describes the technological advancements that led to the creation of the printing press.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>It contrasts the impact of the printing press with other factors in the spread of knowledge.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>The word 'reluctant' in the passage is supported by context clues such as the scientist's initial hesitation to share her findings with the public, which aligns with the meaning of 'hesitant' rather than the other options.</t>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>The passage contrasts the impact of the printing press with other factors such as the rise of universities and improved transportation, highlighting a progression of ideas and a rhetorical move of contrast.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>d0a88186-5c3d-420c-bca7-59a6e1f0bd4d</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Words in Context</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Text Structure</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The city’s library, once considered obsolete, has experienced a remarkable transformation. In recent years, it has not only increased its collection of digital books but also introduced community programs and technology workshops. This evolution has made the library indispensable to residents. No longer just a place for borrowing books, it has become a vibrant hub where people gather to learn and connect. The change from being overlooked to being essential demonstrates how institutions can adapt to meet the changing needs of society.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>For centuries, historians have asserted that the fall of ancient civilizations was primarily due to external invasions. This viewpoint emphasizes the destructive impact of hostile forces overwhelming established societies. However, recent scholarship suggests a more nuanced interpretation. Instead of attributing collapse solely to outside threats, some experts now highlight internal weaknesses—such as political instability and resource depletion—as significant contributing factors. Thus, while external invasions were undoubtedly influential, it is essential to consider the complex interplay of internal and external dynamics when analyzing the decline of ancient societies.</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>In the passage, what does the word 'indispensable' most nearly mean?</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Irrelevant</t>
+          <t>How does the passage develop its argument about the fall of ancient civilizations?</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Essential</t>
+          <t>By providing statistical evidence to support the role of external invasions.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>By describing the political systems of ancient civilizations in detail.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Temporary</t>
+          <t>By contrasting traditional and recent perspectives on the causes of decline.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>By emphasizing the role of resource depletion over external threats.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>The passage describes how the library has become an essential part of the community, indicating that 'indispensable' means 'essential'.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>The passage contrasts the traditional view that external invasions were the primary cause of collapse with recent scholarship that suggests internal factors also played a significant role, demonstrating a shift in understanding.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>f92d087d-be6e-4880-bf7e-1a9c7cd7bb4d</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Words in Context</t>
-        </is>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Text Structure</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Many animals migrate to survive seasonal changes. For instance, birds often embark on long journeys to find warmer climates and abundant food. The word 'embark' means to begin or start something important, especially a journey. These annual trips are challenging, yet essential. Without migration, many species would struggle to obtain enough resources during harsh winters. Thus, migration is not just a choice, but a necessity for survival.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>For centuries, historians have posited that the fall of ancient civilizations was primarily the consequence of external invasions or catastrophic environmental changes. Proponents of this view cite archaeological evidence of abrupt population decline following natural disasters or military incursions. However, a growing body of scholarship challenges this singular perspective by emphasizing the role of internal socio-political dynamics. Specifically, researchers now argue that endemic corruption, administrative inefficiency, and civil unrest often precipitated decline long before external threats materialized. Thus, while external factors cannot be dismissed entirely, it is increasingly apparent that internal vulnerabilities frequently set the stage for collapse.</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>In the context of the passage, what does the word 'embark' most nearly mean?</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>begin</t>
+          <t>How does the passage develop its argument regarding the fall of ancient civilizations?</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>avoid</t>
+          <t>By describing the cultural achievements of ancient civilizations before their fall.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>delay</t>
+          <t>By listing external factors as the primary reasons for the collapse.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>end</t>
+          <t>By providing a chronological timeline of events leading to the fall of civilizations.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>By contrasting the traditional view with a newer perspective on the causes of decline.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>The passage defines 'embark' as to begin or start something important, especially a journey. The context of birds starting long journeys supports this meaning.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>The passage develops its argument by contrasting the traditional view that emphasizes external invasions or environmental changes with a newer perspective that highlights internal socio-political dynamics as primary causes of decline.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>d24d63c5-84fe-4445-972c-ff08e0af229b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Words in Context</t>
-        </is>
-      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Cross-Text</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>While the term 'innovation' is frequently associated with groundbreaking technological advances, its meaning extends beyond mere novelty. In the context of scientific research, innovation often refers to the gradual refinement of existing theories or methods. This incremental progress, although less conspicuous than dramatic discoveries, is indispensable to the advancement of knowledge. Thus, to equate innovation solely with spectacular breakthroughs is to overlook the subtle yet critical improvements that drive scientific achievement.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Text 1: Some historians argue that the printing press was the most important invention of the Renaissance because it allowed ideas to spread quickly and widely. They emphasize that books became more affordable, which helped more people learn to read and share information. 
+Text 2: However, other scholars point out that the printing press alone did not cause these changes. They suggest that improvements in paper making and rising interest in education also played key roles. According to this view, the printing press was one part of a larger movement that transformed society.</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>In the passage, what does the word 'novelty' most nearly mean?</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>newness</t>
+          <t>How do the two texts differ in their perspective on the impact of the printing press during the Renaissance?</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>complexity</t>
+          <t>Text 1 views the printing press as the sole factor in spreading ideas, while Text 2 sees it as part of a broader movement.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>tradition</t>
+          <t>Text 1 suggests the printing press was important for education, while Text 2 focuses on its economic impact.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>simplicity</t>
+          <t>Text 1 argues that the printing press had little impact, whereas Text 2 believes it was crucial.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
+          <t>Text 1 highlights improvements in paper making, whereas Text 2 does not mention it.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>The word 'novelty' in the passage is used in the context of contrasting with 'groundbreaking technological advances' and 'incremental progress,' which suggests that 'novelty' refers to something new or innovative. Thus, 'newness' is the most appropriate interpretation.</t>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Text 1 emphasizes the printing press as the most important invention for the spread of ideas, whereas Text 2 suggests it was only one part of a larger societal transformation.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>aa3f76eb-dca1-46e4-96f1-7081d812f065</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Words in Context</t>
-        </is>
-      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Cross-Text</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Although the historian’s account initially exudes an air of certitude, a closer examination reveals that her conclusions are, in fact, provisional. She meticulously assembles an array of primary sources, yet she repeatedly employs qualifiers such as 'likely' and 'presumably.' This linguistic caution suggests that her assertions, rather than being definitive, are tentative extrapolations based on incomplete evidence. The use of such measured language underscores her recognition of the inherent ambiguities present in reconstructing past events, thereby inviting readers to appreciate the complexity rather than the finality of historical interpretation.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Text 1: Many historians assert that technological innovation consistently drives societal progress, as new inventions often reshape economies and daily life. For example, the printing press not only revolutionized communication but also contributed to the spread of literacy and the acceleration of scientific discovery. This perspective emphasizes the transformative power of technology as a principal catalyst for historical change.
+Text 2: While technological advances undeniably influence societies, some scholars argue that cultural values and social structures frequently determine the impact of these innovations. The printing press, for instance, had varying effects depending on a region's existing educational systems and openness to new ideas. Thus, the significance of technological change is often shaped by the context in which it occurs, rather than by the invention alone.</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>In the context of the passage, what does the word 'provisional' most nearly mean?</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>unnecessary</t>
+          <t>How do the two texts differ in their views on the role of technology in societal change?</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>temporary</t>
+          <t>Text 1 believes that technology affects all societies equally, while Text 2 argues it varies by region.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>permanent</t>
+          <t>Text 1 sees technology as the main driver of change, while Text 2 emphasizes the influence of cultural and social factors.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>definite</t>
+          <t>Text 1 focuses on economic impacts, while Text 2 discusses cultural impacts.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
+          <t>Text 1 argues that technology has a negative impact, whereas Text 2 suggests it is mostly positive.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>The passage indicates that the historian's conclusions are 'provisional' as she uses qualifiers and acknowledges the complexities and ambiguities in reconstructing past events, suggesting that her conclusions are not final or permanent. Thus, 'provisional' most nearly means 'temporary'.</t>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Text 1 emphasizes the transformative power of technology as a principal catalyst for historical change, while Text 2 argues that the significance of technological change is shaped by cultural values and social structures.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>0b627c32-2618-4f9e-a6d1-bfb59a18b8d6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Craft and Structure</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Text Structure</t>
-        </is>
-      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Cross-Text</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>For many years, researchers believed that honeybees only communicated through simple buzzing sounds. According to this view, bees made noises to alert others of danger or to signal their presence. However, recent studies have revealed a more complex form of communication. In fact, scientists have discovered that honeybees use a special 'waggle dance' to share information about the location of food sources. This surprising discovery suggests that honeybee communication is much more advanced than previously thought.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Text 1: Some historians argue that the Industrial Revolution was predominantly a consequence of technological ingenuity, contending that the proliferation of inventions such as the steam engine catalyzed profound economic and social transformations. This perspective underscores the primacy of individual innovators in driving systemic change, often minimizing the role of existing social structures.
+Text 2: While acknowledging the significance of technological advances, other scholars assert that the Industrial Revolution's momentum derived chiefly from shifts in societal organization, such as the rise of urban labor markets and the expansion of financial institutions. By emphasizing these structural factors, this view reframes technological innovation as a product, rather than a cause, of broader economic and social developments.</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>How does the passage develop the idea of honeybee communication?</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>By describing the visual aspects of the waggle dance.</t>
+          <t>What is the primary difference in how the two texts attribute the cause of the Industrial Revolution?</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>By listing various forms of communication used by honeybees.</t>
+          <t>Text 1 attributes it mainly to technological ingenuity, while Text 2 attributes it mainly to shifts in societal organization.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>By contrasting previous beliefs with new research findings.</t>
+          <t>Text 1 attributes it mainly to social structures, while Text 2 attributes it mainly to individual innovators.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>By providing a chronological history of honeybee studies.</t>
+          <t>Text 1 attributes it mainly to financial institutions, while Text 2 attributes it mainly to urban labor markets.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Text 1 attributes it mainly to economic policies, while Text 2 attributes it mainly to technological advances.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>The passage starts with previously held beliefs about honeybee communication and introduces new research findings that contradict those beliefs, highlighting the contrast between old and new understanding.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Text 1 emphasizes the role of technological ingenuity and individual innovators, while Text 2 emphasizes shifts in societal organization, such as urban labor markets and financial institutions, as the primary drivers of the Industrial Revolution.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Craft and Structure</t>
+          <t>887c098a-d472-4ead-b0d4-96befb6c12d1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Text Structure</t>
+          <t>Information and Ideas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Central Idea</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Many historians assert that the invention of the printing press in the fifteenth century was the single most transformative event in the spread of knowledge. They argue that the ability to produce books quickly and in large quantities revolutionized education, empowered new voices, and accelerated the flow of ideas throughout Europe. However, it is important to consider that the printing press alone did not guarantee widespread literacy or access to information. In fact, social and economic barriers continued to limit who could read and own books for centuries. Thus, while the printing press was undoubtedly significant, its impact must be understood within the broader context of gradual social change.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Honey bees are essential to many natural and agricultural systems. By moving from flower to flower in search of nectar, they carry pollen that helps plants reproduce. This process, called pollination, leads to the production of fruits, vegetables, and seeds. Without honey bees, many of the foods people rely on would become much less available. In addition to their role in pollination, honey bees also produce honey, which has been valued by humans for centuries. Their impact on both ecosystems and human diets makes honey bees an important species worldwide.</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>How does the author structure the passage to present the impact of the printing press?</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>By listing the technological advancements that accompanied the printing press.</t>
+          <t>Which choice best states the main idea of the passage?</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>By contrasting the immediate effects with the long-term societal changes.</t>
+          <t>Without pollination, fruits and vegetables would not be as abundant.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>By comparing the printing press to other historical inventions.</t>
+          <t>Honey bees are crucial for both pollination and honey production, impacting ecosystems and human diets.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>By providing a chronological history of the printing press's invention.</t>
+          <t>Honey bees only play an important role in the pollination of agricultural systems.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
+          <t>Honey production is the most significant contribution of honey bees to human society.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>The passage contrasts the immediate transformative effects of the printing press with the ongoing social and economic limitations that affected its impact over time, indicating a structure that highlights both immediate and gradual changes.</t>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>The passage discusses the essential role of honey bees in pollination and honey production, emphasizing their importance to ecosystems and human diets. Option A synthesizes these points as the central idea of the passage.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Craft and Structure</t>
+          <t>066981ad-f22e-4a7d-ac97-04335748efd7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Text Structure</t>
+          <t>Information and Ideas</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Central Idea</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>For centuries, historians posited that the collapse of the ancient Maya civilization was precipitated primarily by protracted drought. This interpretation, grounded in paleoclimatic data and supported by archaeological findings, dominated scholarly discourse. However, recent research has introduced a competing hypothesis: that internal sociopolitical instability played an equally significant role. While environmental stressors undeniably strained resources, proponents of this newer perspective contend that escalating warfare, leadership fragmentation, and unequal resource distribution critically undermined the resilience of Maya society. Thus, rather than attributing the decline to a single cause, contemporary scholars increasingly advocate for a multifactorial model, emphasizing the interplay between environmental and human factors.</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Throughout the twentieth century, the development of antibiotics dramatically changed the treatment of infectious diseases. Before their introduction, illnesses such as pneumonia and tuberculosis often proved fatal, with few effective remedies available. However, the widespread use of antibiotics led to a sharp decline in deaths from these conditions. Despite these gains, medical experts have observed that overuse and misuse of antibiotics have contributed to the emergence of resistant bacteria, prompting renewed concerns about the future effectiveness of these life-saving drugs.</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>How does the passage structure the presentation of ideas regarding the collapse of the ancient Maya civilization?</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>It lists various environmental factors leading to the collapse.</t>
+          <t>Which choice best describes the central claim of the passage?</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>It focuses on the role of external invasions in the collapse.</t>
+          <t>The introduction of antibiotics was a significant medical advancement in the fight against infectious diseases.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>It contrasts two hypotheses about the causes of the collapse.</t>
+          <t>Medical experts are worried about the misuse of antibiotics, which could render them ineffective in the future.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>It describes the chronological sequence of the civilization's decline.</t>
+          <t>The development of antibiotics has drastically reduced deaths from infectious diseases but has led to concerns about antibiotic resistance.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
+          <t>Antibiotics were not available before the twentieth century, making diseases like pneumonia and tuberculosis often fatal.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>The passage begins by presenting the traditional hypothesis that attributes the collapse to drought. It then introduces a competing hypothesis, emphasizing internal sociopolitical factors, and concludes by advocating for a multifactorial model. This structure highlights the contrast between the two perspectives.</t>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Option A synthesizes the main idea by highlighting both the positive impact of antibiotics and the ongoing concerns about resistance, which is the central focus of the passage.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Craft and Structure</t>
+          <t>4ebc9c36-d10e-45ab-a7cc-5954b000f47b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cross-Text</t>
+          <t>Information and Ideas</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Central Idea</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Text 1: Historians often describe the invention of the printing press as a turning point in human communication. Before its introduction, books were rare and copying texts by hand was slow and expensive. The printing press made it possible to produce many copies quickly, allowing ideas to spread rapidly across countries and cultures. 
-Text 2: While the printing press certainly increased the number of books available, some historians point out that the change took time. Many people could not read, and books remained expensive for years after printing began. This suggests that the impact of the printing press depended not only on the technology itself, but also on social and economic conditions.</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>In the early nineteenth century, the introduction of steam locomotives dramatically altered patterns of economic development and social mobility in Britain. Railways enabled manufacturers to ship goods swiftly over long distances, reducing costs and expanding markets far beyond local regions. At the same time, easier travel encouraged populations to migrate from rural areas to industrial cities, fueling urban growth and reshaping demographic structures. These shifts, however, also contributed to the decline of traditional crafts and local economies, as small-scale producers found it increasingly difficult to compete. Thus, while the railway network fostered national integration and modernization, it also generated profound disruptions to established ways of life.</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>How do the two texts differ in their portrayal of the impact of the printing press?</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Text 1 focuses on the technological innovation, while Text 2 discusses the decline of handwritten texts.</t>
+          <t>Which choice best describes the central claim of the passage?</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Text 1 and Text 2 both agree that the printing press made books affordable immediately.</t>
+          <t>Steam locomotives primarily benefited manufacturers by reducing shipping costs and expanding markets.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Text 1 emphasizes the immediate spread of ideas, while Text 2 highlights the gradual nature of this change.</t>
+          <t>The railway network in Britain led to national integration and modernization, despite causing disruptions to traditional ways of life.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Text 1 argues that the printing press had no significant impact, while Text 2 illustrates its importance.</t>
+          <t>The decline of traditional crafts was the most significant impact of the railway network.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Urban growth and demographic changes were the direct results of easier travel provided by railways.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Text 1 describes the printing press as a turning point that quickly allowed ideas to spread, while Text 2 suggests the impact was slower due to literacy and economic factors.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Option A captures the main idea of the passage, which describes how the railway network in Britain drove national integration and modernization while also causing significant disruptions to established ways of life. Other options focus on narrower aspects of the passage or secondary effects.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Craft and Structure</t>
+          <t>b7ad9f14-d9e8-49f6-a747-4fbb6d1203de</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cross-Text</t>
+          <t>Information and Ideas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Command of Evidence</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Text 1: Some historians argue that technological innovation is primarily a response to societal needs, suggesting that every major invention reflects the challenges faced by a particular era. According to this perspective, the steam engine arose out of the necessity for efficient transportation during the Industrial Revolution, rather than from scientific curiosity alone.
-Text 2: While societal needs undeniably shape technological progress, other historians contend that innovation often precedes demand, transforming society in unexpected ways. For instance, the development of personal computers did not respond to a widespread, articulated need, but instead created new possibilities and ultimately altered daily life and work patterns.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Some historians argue that bicycles played an important role in expanding personal freedom during the late 1800s. Unlike trains, which followed fixed routes and schedules, bicycles allowed individuals to travel independently at any time. Many people found that owning a bicycle meant they could visit friends or commute to work more easily. Newspapers from that era reported that even women, who often had limited mobility, began to use bicycles for daily tasks. The popularity of bicycles also encouraged the improvement of roads, making travel safer and more accessible for everyone.</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>How do the authors of Text 1 and Text 2 differ in their views on the relationship between societal needs and technological innovation?</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Text 1 suggests that technological innovation is driven by societal needs, while Text 2 suggests that innovation can occur independently of immediate demand.</t>
+          <t>Which detail from the passage best supports the claim that bicycles expanded personal freedom in the late 1800s?</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Text 1 believes that societal needs always follow technological innovation, whereas Text 2 believes they precede it.</t>
+          <t>Bicycles allowed individuals to travel independently at any time.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Text 1 argues that scientific curiosity is the primary driver of innovation, while Text 2 argues that societal needs are more influential.</t>
+          <t>The popularity of bicycles also encouraged the improvement of roads.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Text 1 claims that technological advances always transform society, while Text 2 claims they rarely have an impact.</t>
+          <t>Newspapers from that era reported that even women began to use bicycles for daily tasks.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
+          <t>Many people found that owning a bicycle meant they could visit friends or commute to work more easily.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Text 1 emphasizes that technological innovation, like the steam engine, arises from societal needs, while Text 2 highlights that innovation, like personal computers, can occur without a pre-existing demand, suggesting a contrast in views.</t>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Option A directly supports the claim by highlighting the independent travel capability of bicycles, which is central to the idea of expanding personal freedom.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Craft and Structure</t>
+          <t>44452154-4d6f-448a-bd34-bc5ea8303e74</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cross-Text</t>
+          <t>Information and Ideas</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Command of Evidence</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Text 1: Some historians argue that technological innovation inherently accelerates social progress, suggesting that advancements such as the printing press or the internet democratize knowledge and catalyze reform. These scholars emphasize the direct causal relationship between new tools and the restructuring of societal hierarchies. 
-Text 2: However, others contend that the influence of technology is contingent upon preexisting cultural and institutional frameworks. For example, the diffusion of the printing press in fifteenth-century Europe yielded disparate effects depending on local governance and literacy rates, indicating that technology’s impact is mediated by the context into which it is introduced.</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>In the early 20th century, city planners began to recognize the importance of public parks for urban communities. Some officials believed that green spaces promoted physical health by encouraging outdoor activities, while others argued that parks improved mental well-being by providing a peaceful environment. Reports from the period indicate that neighborhoods with access to parks experienced lower rates of certain illnesses and higher community satisfaction. Although some critics questioned the cost of maintaining these areas, surveys consistently showed that residents valued public parks highly.</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>How do the two texts differ in their views on the role of technology in social progress?</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Text 1 claims that technology has no effect on social progress, whereas Text 2 believes it accelerates change.</t>
+          <t>Which detail from the passage best supports the claim that public parks were valued by urban communities in the early 20th century?</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Text 1 argues that technology directly causes societal change, while Text 2 suggests its effects are dependent on existing conditions.</t>
+          <t>Although some critics questioned the cost of maintaining these areas.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Text 1 focuses on the negative impacts of technology, while Text 2 highlights its positive contributions.</t>
+          <t>Reports from the period indicate that neighborhoods with access to parks experienced lower rates of certain illnesses.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Text 1 and Text 2 both agree that technology always leads to positive social progress.</t>
+          <t>Some officials believed that green spaces promoted physical health.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Surveys consistently showed that residents valued public parks highly.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Text 1 suggests a direct causal relationship between technological innovation and social progress, whereas Text 2 emphasizes the mediating role of preexisting cultural and institutional frameworks.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Option A directly supports the claim by stating that surveys showed residents valued parks highly, indicating their appreciation and perceived importance of these spaces.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>8f8b7941-799a-4dbc-8cd4-15370d5a0e4a</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Central Idea</t>
-        </is>
-      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Command of Evidence</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Honeybees play a vital role in pollinating many of the crops that people rely on for food. As they move from flower to flower collecting nectar, they transfer pollen, which helps plants produce fruit and seeds. In recent years, scientists have noticed a decline in honeybee populations, raising concerns about the impact this could have on agriculture. Protecting honeybees is important not just for the bees themselves, but also for the health of ecosystems and the food supply.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Although the introduction of the printing press in fifteenth-century Europe is often credited with revolutionizing the spread of information, its immediate effects were uneven across the continent. In regions with established urban centers and high literacy rates, such as parts of Germany and Italy, printed books rapidly supplanted handwritten manuscripts and facilitated the exchange of scientific and philosophical ideas. However, in rural or politically fragmented areas, manuscript culture persisted for decades, and the accessibility of printed works remained limited. Nevertheless, the eventual proliferation of affordable printed materials is widely believed to have played a significant role in the acceleration of the Renaissance and the Reformation.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Which choice best states the main idea of the passage?</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Scientists have observed a decline in honeybee populations in recent years.</t>
+          <t>Which detail from the passage best supports the claim that the introduction of the printing press had uneven immediate effects across Europe?</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Honeybees collect nectar from flowers to produce fruit and seeds.</t>
+          <t>The accessibility of printed works remained limited in some areas.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Protecting honeybees is important for maintaining biodiversity.</t>
+          <t>The eventual proliferation of affordable printed materials is believed to have accelerated the Renaissance and the Reformation.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Honeybees are essential for pollinating crops and their decline raises concerns for agriculture.</t>
+          <t>In rural or politically fragmented areas, manuscript culture persisted for decades.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>In regions with established urban centers and high literacy rates, such as parts of Germany and Italy, printed books rapidly supplanted handwritten manuscripts.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>The passage centers on the importance of honeybees in pollination and the potential agricultural impact of their decline, making option A the best summary of the main idea.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Option B directly supports the claim of uneven immediate effects by highlighting how manuscript culture persisted in less developed areas, contrasting with regions where printed books quickly supplanted manuscripts.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>5be76f78-eef6-4a76-9670-2574691eea17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Central Idea</t>
-        </is>
-      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Inference</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>In the early twentieth century, city planners began to recognize the importance of public parks in urban environments. These green spaces were not only designed for recreation but also served as vital areas for improving public health and fostering social interaction. By providing residents with access to nature and opportunities for exercise, parks were believed to counteract some negative effects of dense city living. Over time, research continued to affirm the value of parks, leading many cities to invest in expanding and maintaining these spaces as essential components of urban life.</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Over the past decade, the city park has seen a significant increase in the number of visitors during weekends. Local officials have responded by adding more benches and expanding the playground area. Despite these improvements, maintenance reports show that the park's grassy areas are wearing down faster each year. City planners are now discussing ways to encourage visitors to use designated walking paths more often.</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Which choice best states the main idea of the passage?</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>City planners in the early twentieth century focused solely on recreation when designing parks.</t>
+          <t>Which inference is best supported by the passage?</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Urban environments are negatively affected by dense city living.</t>
+          <t>Local officials are trying to balance increased park usage with maintaining the park's condition.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Public parks play a crucial role in enhancing urban life by improving health and social interaction.</t>
+          <t>Visitors prefer grassy areas over walking paths during weekdays.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Many cities have invested in parks due to research findings.</t>
+          <t>The city plans to replace all grassy areas with walking paths to prevent wear.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>The addition of benches and playground space has led to fewer visitors using walking paths.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>The passage highlights the importance of public parks in urban settings, emphasizing their role in improving health and fostering social interaction, which aligns with option A. Other options are either too narrow, too broad, or focus on secondary details.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>The passage discusses the increase in park visitors and the resulting wear on grassy areas, along with the officials' response of adding benches and playgrounds while considering ways to encourage path use, suggesting an effort to balance usage with maintenance.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>914cd348-a61c-48ba-99d8-e4fb156c0ad6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Central Idea</t>
-        </is>
-      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Inference</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>During the nineteenth century, the proliferation of railroads dramatically altered patterns of economic activity across continents. Previously isolated regions became integrated into broader markets, enabling producers to sell goods far from their point of origin. In addition, the rapid movement of raw materials and finished products fostered the expansion of industries and urban centers. However, these benefits were not distributed evenly; communities bypassed by railway lines often experienced economic stagnation or decline, underscoring the transformative but uneven nature of technological progress.</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>In the early twentieth century, several American cities began to implement strict zoning laws, regulating where businesses and homes could be built. Proponents argued that separating industrial and residential areas would improve public health by reducing residents’ exposure to pollution. However, critics noted that these laws often resulted in low-income families being concentrated in less desirable neighborhoods, farther from job opportunities and city services. Over time, some cities modified their zoning policies, aiming to balance economic growth with equitable access to resources.</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Which choice best describes the central idea of the passage?</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>The expansion of railroads in the nineteenth century transformed economic activities but led to unequal benefits.</t>
+          <t>What can be most reasonably inferred about the effect of early zoning laws on low-income families?</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Railroads primarily benefited urban centers by facilitating the movement of goods.</t>
+          <t>They benefited from reduced exposure to pollution due to residential zoning.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Isolated regions failed to integrate into broader markets due to the lack of railroads.</t>
+          <t>They experienced improved access to city services and economic growth.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Technological advancements in transportation always result in economic growth.</t>
+          <t>They were able to live closer to industrial areas, improving their job prospects.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>They were often forced to live in less desirable areas farther from job opportunities.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>The passage discusses how railroads altered economic activities and integrated regions into markets while also noting that the benefits were not evenly distributed, which aligns with option A as the central idea.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>The passage discusses how zoning laws often resulted in low-income families being concentrated in less desirable neighborhoods, farther from job opportunities and city services, allowing for an inference that they were negatively impacted by these laws.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>a94b0e3b-2367-429e-8b1d-2a4533930157</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Command of Evidence</t>
-        </is>
-      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Inference</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>During the early 20th century, cities in the United States experienced significant growth. Many people moved from rural areas to urban centers in search of employment. Factories in cities offered more job opportunities than farms, especially as new industries developed. This shift contributed to rising urban populations. As a result, city governments expanded public services such as transportation and sanitation to accommodate the increasing number of residents.</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>In the early 20th century, several Arctic expeditions reported that the region’s sea ice extended farther south than previously recorded. However, by the 1940s, navigators began noting increased seasonal variability in ice coverage, with some routes opening earlier in the year. Despite improvements in navigation and ship technology, accounts from this period still emphasized the unpredictability of ice conditions, often attributing it to shifting winds and temperatures. These observations were made decades before the advent of satellite monitoring, relying instead on direct encounters and logbooks maintained by crews.</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Which detail from the passage best supports the conclusion that urbanization led to changes in city infrastructure?</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>This shift contributed to rising urban populations.</t>
+          <t>What can be inferred about Arctic sea ice conditions in the early to mid-20th century based on the passage?</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Many people moved from rural areas to urban centers in search of employment.</t>
+          <t>Satellite monitoring was the main tool for studying Arctic sea ice in the early 20th century.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Factories in cities offered more job opportunities than farms.</t>
+          <t>Arctic sea ice conditions were unpredictable despite advancements in technology.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>City governments expanded public services such as transportation and sanitation.</t>
+          <t>Ice coverage consistently decreased throughout the 20th century.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Shifting winds and temperatures had no impact on sea ice conditions.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Option A directly addresses how city infrastructure had to adapt to support the growing urban population, making it the strongest evidence for the conclusion about changes in city infrastructure due to urbanization.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>The passage discusses the unpredictability of ice conditions and mentions that this unpredictability was noted despite technological improvements, supporting the inference that Arctic sea ice conditions were unpredictable.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>27f602dd-e102-45f3-82b8-ab348cf219fe</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Command of Evidence</t>
-        </is>
-      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Data Interpretation</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>In recent years, urban planners have increasingly promoted the development of green roofs as a strategy to address the environmental challenges faced by cities. Green roofs, which consist of vegetation planted atop buildings, are believed to reduce stormwater runoff by absorbing rainwater that would otherwise flow into city sewers. In addition, some studies suggest that green roofs help to lower urban temperatures by providing shade and releasing moisture into the air. While the installation of green roofs can be costly, advocates argue that the long-term benefits, such as improved air quality and reduced energy use, outweigh the initial expenses.</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A recent study examined the reading habits of middle school students in two cities. In City A, 60% of students reported reading for pleasure at least once a week, while in City B, only 40% did so. Over a one-year period, students in City A read an average of 12 books each, compared to an average of 7 books per student in City B. The researchers also found that the percentage of students who reported enjoying reading increased by 10% in City A but remained unchanged in City B.</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Which detail from the passage best supports the claim that green roofs are beneficial in urban environments?</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Advocates argue that the long-term benefits outweigh the initial expenses.</t>
+          <t>Which conclusion is best supported by the data reported in the passage regarding the reading habits of students in City A and City B?</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>The installation of green roofs can be costly.</t>
+          <t>The number of books read by students in City A decreased over the one-year period.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Some studies suggest that green roofs help to lower urban temperatures.</t>
+          <t>Students in City A are more likely to read for pleasure compared to students in City B.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Green roofs are believed to reduce stormwater runoff by absorbing rainwater.</t>
+          <t>The enjoyment of reading decreased in City B over the one-year period.</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Students in City B read more books on average than students in City A.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Option A directly supports the claim about the benefit of green roofs by explaining how they reduce stormwater runoff, which is a significant environmental challenge in urban areas. While options B and D also mention benefits, option A provides a specific mechanism of how green roofs contribute to urban environmental improvement.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>The passage states that 60% of students in City A reported reading for pleasure at least once a week, compared to 40% in City B. This supports the conclusion that students in City A are more likely to read for pleasure.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>c829a182-23b4-435b-84b1-204a5bb62fe7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Command of Evidence</t>
-        </is>
-      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Data Interpretation</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Although many historians once attributed the rapid urbanization of late 19th-century cities primarily to industrial job opportunities, recent analyses suggest a more complex interplay of factors. While factories did attract rural laborers, municipal investments in public transportation and housing infrastructure also played a critical role in facilitating population growth. For instance, the expansion of streetcar lines enabled workers to reside farther from industrial centers, thereby dispersing dense inner-city populations. Additionally, city governments implemented public health measures, such as waste management systems, which reduced disease incidence and made urban life more sustainable. These developments collectively indicate that urbanization during this period was driven not solely by employment prospects but also by deliberate urban planning and public policy interventions.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>A recent study examined the reading habits of 500 high school students over a two-month period. Researchers found that 68% of students read for at least 30 minutes each day, while 22% read for less than 15 minutes daily. Only 10% reported not reading at all outside of school assignments. Compared to the previous year, the proportion of daily readers increased by 8 percentage points, while the percentage of students who did not read outside of school decreased by 5 percentage points.</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Which detail from the passage best supports the claim that urbanization in the late 19th century was influenced by factors other than employment opportunities?</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>City governments implemented public health measures to reduce disease incidence.</t>
+          <t>Which conclusion is best supported by the reported results about the change in students' reading habits over the past year?</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Municipal investments in public transportation facilitated population growth.</t>
+          <t>More students are reading daily compared to the previous year.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Factories attracted rural laborers to urban areas.</t>
+          <t>Fewer students are reading outside of school assignments compared to the previous year.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Streetcar lines enabled workers to reside farther from industrial centers.</t>
+          <t>The proportion of students who do not read at all has remained the same.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>The percentage of students who read for less than 15 minutes daily has decreased.</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Option A directly supports the claim by highlighting the role of municipal investments, which is a factor other than employment opportunities. Other options either focus on employment (D) or provide examples of how urban life was made more sustainable (B, C), but do not directly address the broader influence beyond jobs.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>The passage states that the proportion of daily readers increased by 8 percentage points compared to the previous year, indicating more students are reading daily.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>ce379b78-d55b-4a97-b0d0-1811cbaaeca3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>Information and Ideas</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Inference</t>
-        </is>
-      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Data Interpretation</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>In the early 1900s, most city streets were crowded with horses pulling carriages and carts. These animals required daily care, including feeding and cleaning. When motor vehicles began to appear, they were at first considered unreliable and noisy. However, over time, more people purchased automobiles, and the number of horses in cities declined. By the 1920s, it was rare to see a horse on a busy city street.</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A longitudinal study examined the cognitive performance of adults aged 50 to 75 over a ten-year period. At the outset, participants were divided into two groups based on their engagement in mentally stimulating activities: Group A (those who engaged in such activities weekly) and Group B (those who did so infrequently, less than once a month). After ten years, Group A exhibited an average decline in cognitive test scores of 7%, whereas Group B experienced a decline of 18%. Furthermore, while 12% of individuals in Group A showed no significant decline, only 3% of Group B maintained stable scores. These findings persisted even after controlling for variables such as education and physical health.</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>The passage most strongly suggests that the decline in the number of horses on city streets was primarily due to:</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>a lack of daily care for horses in cities.</t>
+          <t>Which conclusion is best supported by the reported results of the study?</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>the increasing reliability and popularity of motor vehicles.</t>
+          <t>Engaging in mentally stimulating activities frequently is associated with a smaller decline in cognitive performance.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>the rapid decline in horse population due to disease.</t>
+          <t>Cognitive performance in adults is primarily determined by physical health.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>the complaints about the noise created by motor vehicles.</t>
+          <t>The decline in cognitive performance is unavoidable for all adults over time.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Education level is the most significant factor in maintaining cognitive stability.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>The passage implies that as motor vehicles grew in popularity and were purchased by more people, horses became less common on city streets. This suggests that the shift from horse-drawn carriages to motor vehicles was a primary factor in the decline of horses in urban areas.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>The passage describes that Group A, who engaged in mentally stimulating activities weekly, had a smaller average decline in cognitive test scores compared to Group B, who did so infrequently. This supports the conclusion that frequent engagement in such activities is associated with a smaller decline.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Information and Ideas</t>
+          <t>ff45289b-4341-4fe7-94c9-e7c6b4723b94</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Inference</t>
+          <t>Standard English Conventions</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Boundaries</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>During the early stages of the Industrial Revolution, many textile factories were constructed near rivers. Factory owners often recruited workers from distant rural areas, providing them with basic lodging close to the mills. Workers frequently labored for long hours, and letters from the period mention fatigue and a lack of time for personal pursuits. Nonetheless, some owners reported high rates of worker retention from season to season, which they attributed to the relative scarcity of alternative employment in the surrounding countryside.</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Marie Curie conducted groundbreaking research in radioactivity however, her achievements were not fully recognized during her lifetime.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Marie Curie conducted groundbreaking research in radioactivity however, her achievements were not fully recognized during her lifetime.</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>What can be most reasonably inferred about the workers' decision to stay at the textile factories from one season to another?</t>
+          <t>however,</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Workers primarily stayed due to strong community ties within the factory.</t>
+          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Workers were satisfied with the wages and working conditions at the factories.</t>
+          <t>however, her</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Workers had limited job opportunities in their local rural areas.</t>
+          <t>however; her</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Workers were required to stay for multiple seasons by contract.</t>
+          <t>however. Her</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>however her,</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>The passage mentions that factory owners reported high retention rates attributed to a scarcity of alternative employment, suggesting that workers stayed due to limited job options.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>The correct punctuation to join two independent clauses in this context is to use a semicolon. Option A correctly uses the semicolon to link the clauses 'Marie Curie conducted groundbreaking research in radioactivity' and 'her achievements were not fully recognized during her lifetime.'</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Information and Ideas</t>
+          <t>1d645f66-8e69-4941-b477-a5aed2f896b9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Inference</t>
+          <t>Standard English Conventions</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Boundaries</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>In the early twentieth century, urban planners in several major cities advocated for the creation of public parks, citing the need for green spaces amidst increasing industrialization. Reports from the period reveal that residential districts located closer to these parks experienced a modest but consistent rise in property values over two decades, whereas similarly situated neighborhoods without park access did not. At the same time, city health officials documented a gradual decrease in respiratory ailments among residents living near the new parks, attributing the trend to improved air quality. Although the planners’ initial proposals made little mention of economic benefits or public health, the subsequent changes in these areas suggest broader effects than originally anticipated.</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Researchers conducted several trials to test the new material however, the results were inconclusive.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Researchers conducted several trials to test the new material however, the results were inconclusive.</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Which inference is best supported by the passage?</t>
+          <t>however,</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>City health officials had anticipated the decline in respiratory ailments before the parks were built.</t>
+          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Urban planners underestimated the potential benefits of public parks in their initial proposals.</t>
+          <t>: however,</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Public parks were primarily created to improve air quality in urban areas.</t>
+          <t>, however</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>The increase in property values was the primary goal of the urban planners.</t>
+          <t>however</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>; however,</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>The passage describes how urban planners initially advocated for parks due to industrialization but did not mention economic or health benefits, which were later observed. This implies they underestimated these benefits.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>The correct answer is A because 'however' introduces a new independent clause and should be preceded by a semicolon to properly separate it from the preceding independent clause. Option B lacks necessary punctuation, Option C incorrectly uses a comma, and Option D incorrectly uses a colon.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Information and Ideas</t>
+          <t>4d756108-4eee-41b3-8b20-e294ae4a44f1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Data Interpretation</t>
+          <t>Standard English Conventions</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Boundaries</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>In a study of reading habits among middle school students, researchers found that 60% of students reported reading for pleasure at least once a week. Among these students, 35% read daily, while the remaining 65% read between one and six times per week. The study also noted that students who read daily scored, on average, 10% higher on vocabulary tests compared to those who read less frequently.</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Although the experiment yielded unexpected results, researchers were able to revise their hypothesis; this allowed them to design a more effective follow-up study.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Although the experiment yielded unexpected results, researchers were able to revise their hypothesis; this allowed them to design a more effective follow-up study.</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>According to the passage, which statement is most supported by the data regarding students who read daily?</t>
+          <t>;</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>All students who read daily also read for pleasure at least once a week.</t>
+          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Students who read daily score on average 10% higher on vocabulary tests than those who read less frequently.</t>
+          <t>.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Students who read daily are more likely to read for pleasure at least once a week than those who read less frequently.</t>
+          <t>;</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Daily readers make up 60% of the students who read for pleasure at least once a week.</t>
+          <t>,</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Option A is directly supported by the passage, which states that students who read daily scored, on average, 10% higher on vocabulary tests compared to those who read less frequently. The other options either misinterpret or make unsupported assumptions based on the data provided.</t>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>The semicolon correctly joins two independent clauses in this sentence, showing the relationship between the unexpected results and the revised hypothesis. Other punctuation choices do not correctly join these clauses.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Information and Ideas</t>
+          <t>e3168df2-b72d-49a2-b4af-aab8b2c54595</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Data Interpretation</t>
+          <t>Standard English Conventions</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Form, Structure, and Sense</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>In a study examining reading habits among high school students, researchers found that 62% of participants reported reading for pleasure at least once a week, while 28% read only for school assignments. The remaining 10% reported rarely reading outside of required schoolwork. Over a five-year period, the proportion of students reading for pleasure at least weekly declined by 8 percentage points, while those reading only for school assignments increased by 5 percentage points. Researchers noted that the decline in leisure reading was most pronounced among students in their final year of high school.</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>The scientists in the laboratory measures the temperature of the solution every hour to ensure accuracy.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>The scientists in the laboratory measures the temperature of the solution every hour to ensure accuracy.</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Which conclusion is best supported by the reported data?</t>
+          <t>measures</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Over a five-year period, there was a notable decline in students reading for pleasure at least weekly.</t>
+          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>The majority of high school students read only for school assignments.</t>
+          <t>measures</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Reading habits among high school students have remained constant over the five years.</t>
+          <t>measured</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>All students in their final year of high school stopped reading for pleasure.</t>
+          <t>measure</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>measuring</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Option A is the best supported by the passage as it clearly states that there was a decline in students reading for pleasure at least weekly over a five-year period. Option B is incorrect because it overstates the decline by implying all students stopped reading for pleasure. Option C is incorrect because the data shows that the majority read for pleasure, not just for school. Option D is incorrect because the passage states there were changes in reading habits over the five years.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>The subject 'scientists' is plural, so the verb should also be in the plural form 'measure' to maintain subject-verb agreement.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Information and Ideas</t>
+          <t>ff99df23-40bb-4306-82c6-dd5b8a2ade6e</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Data Interpretation</t>
+          <t>Standard English Conventions</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Form, Structure, and Sense</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>A recent study examined the dietary habits of three age groups: adolescents (ages 12–18), adults (ages 19–64), and seniors (ages 65 and above). Researchers found that 76% of adolescents consumed sugary beverages daily, compared to 51% of adults and 29% of seniors. In contrast, daily fruit intake was reported by only 38% of adolescents, while 62% of adults and 71% of seniors met this guideline. The study also noted that over the past decade, daily sugary beverage consumption declined by 14 percentage points among adults but remained nearly unchanged for adolescents.</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Unlike many other mammals, bats use echolocation to navigate, which allows them to detect obstacles even when ______.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Unlike many other mammals, bats use echolocation to navigate, which allows them to detect obstacles even when ______.</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>According to the passage, which statement is most supported by the reported data regarding sugary beverage consumption?</t>
+          <t>they cannot see them</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Adolescents have shown a significant decrease in sugary beverage consumption over the past decade.</t>
+          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Seniors are less likely to consume sugary beverages daily compared to adolescents and adults.</t>
+          <t>they are not able to see it</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>The majority of seniors do not meet daily fruit intake guidelines.</t>
+          <t>they cannot see it</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Adults consume sugary beverages more frequently than adolescents.</t>
+          <t>they cannot see them</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
+          <t>they do not see it</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>The data in the passage shows that 76% of adolescents, 51% of adults, and 29% of seniors consume sugary beverages daily, which supports that seniors are less likely to consume them than the other groups.</t>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>The correct answer 'they cannot see it' uses the singular pronoun 'it' to refer to the singular noun 'obstacle,' ensuring agreement in number between the pronoun and its antecedent.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>1fdbedc2-2fab-4eb8-b0e8-aca2fe991102</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Boundaries</t>
-        </is>
-      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Form, Structure, and Sense</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Marie Curie conducted groundbreaking research on radioactivity however, she also faced significant obstacles as a woman in science.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Marie Curie conducted groundbreaking research on radioactivity however, she also faced significant obstacles as a woman in science.</t>
+          <t>The committee, along with several of its advisors, _____ planning the conference schedule, but conflicting opinions about the keynote speaker’s role have delayed a final decision.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>however,</t>
+          <t>The committee, along with several of its advisors, _____ planning the conference schedule, but conflicting opinions about the keynote speaker’s role have delayed a final decision.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>is</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>however; she</t>
-        </is>
-      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>however: she</t>
+          <t>is</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>however she</t>
+          <t>were</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>however. She</t>
+          <t>are</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>have been</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>The sentence needs a period after 'radioactivity' to correctly separate the two independent clauses. Option C correctly uses a period to separate the clauses, while options A and D incorrectly use a semicolon and a colon, respectively, and option B incorrectly omits punctuation.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>The subject of the sentence is 'The committee,' which is singular. Therefore, the verb 'is' correctly agrees with the singular subject, making option A the correct choice.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>3bae5d7b-709d-4d50-850c-91e82b2fdfb0</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Boundaries</t>
-        </is>
-      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Modifiers</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Researchers observed an increase in migratory bird populations in the region, however this trend may be temporary as environmental conditions continue to change.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Researchers observed an increase in migratory bird populations in the region, however this trend may be temporary as environmental conditions continue to change.</t>
+          <t>After reading the novel, Maria recommended it to her classmates.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>however</t>
+          <t>After reading the novel, Maria recommended it to her classmates.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>After reading the novel</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>, however</t>
+          <t>Which choice best clarifies the intended meaning while following standard written English?</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>: however</t>
+          <t>After the novel was read,</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>; however,</t>
+          <t>After Maria read the novel,</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>however</t>
+          <t>Reading the novel,</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>After reading the novel,</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>The sentence consists of two independent clauses, which should be properly connected with a semicolon followed by a transitional phrase.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>The correct answer 'After Maria read the novel,' makes it clear that Maria is the one who read the novel, providing proper linkage between the modifier and its intended subject. The other options create ambiguity or misplace the modifier.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>5c6f6065-4735-46c5-be59-17be82deed96</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Boundaries</t>
-        </is>
-      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Modifiers</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>The historian meticulously analyzed the ancient manuscripts, she discovered discrepancies between the recorded events and established timelines.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The historian meticulously analyzed the ancient manuscripts, she discovered discrepancies between the recorded events and established timelines.</t>
+          <t>Climbing rapidly up the steep mountainside, the researchers observed several species of rare plants.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>she discovered</t>
+          <t>Climbing rapidly up the steep mountainside, the researchers observed several species of rare plants.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>Climbing rapidly up the steep mountainside</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>; she discovered</t>
+          <t>Which choice best clarifies the intended meaning while following standard written English?</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>she discovered</t>
+          <t>Having climbed rapidly up the steep mountainside, the researchers</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>and she discovered</t>
+          <t>Climbing rapidly up the steep mountainside, several species of rare plants</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>as she discovered</t>
+          <t>As they climbed rapidly up the steep mountainside, the researchers</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
+          <t>The researchers, who were climbing rapidly up the steep mountainside,</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>The sentence contains two independent clauses that need to be joined with a coordinating conjunction or separated by a semicolon. Option A correctly uses the conjunction 'and' to join the two independent clauses.</t>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Option A correctly places the modifier so that it clearly modifies 'the researchers,' who are the intended subject performing the action of climbing. The other options misplace the modifier, leading to illogical meanings.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>fdd85739-e70d-4e66-aee7-3960bc3a36e1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Form, Structure, and Sense</t>
-        </is>
-      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Modifiers</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Maria and her teammates review the experiment’s results every week and then ___ a summary report for their teacher.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Maria and her teammates review the experiment’s results every week and then ___ a summary report for their teacher.</t>
+          <t>While reviewing the results of the experiment, the unexpected increase in temperature surprised the researchers.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>writes</t>
+          <t>While reviewing the results of the experiment, the unexpected increase in temperature surprised the researchers.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>While reviewing the results of the experiment</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>writing</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>write</t>
+          <t>While reviewing the results of the experiment,</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>writes</t>
+          <t>While the experiment was reviewed,</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>written</t>
+          <t>While the results of the experiment were reviewed,</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>While they were reviewing the results of the experiment,</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>The subject 'Maria and her teammates' is plural, so the correct verb form is 'write' to match the plural subject.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>The original sentence contains a dangling modifier because 'reviewing the results of the experiment' does not clearly modify the subject 'the unexpected increase in temperature.' Option A corrects this by specifying that 'they' (the researchers) are the ones reviewing the results, which logically connects the modifier to its intended subject.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>f4677f55-a468-4396-98ed-e5df171edf8a</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Form, Structure, and Sense</t>
-        </is>
-      </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Punctuation</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>While many scientists agree on the importance of climate research, a significant number of them believes that more funding is necessary to advance the field.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>While many scientists agree on the importance of climate research, a significant number of them believes that more funding is necessary to advance the field.</t>
+          <t>During the Renaissance many artists—including Leonardo da Vinci—explored new techniques in painting and sculpture.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>believes</t>
+          <t>During the Renaissance many artists—including Leonardo da Vinci—explored new techniques in painting and sculpture.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>—including Leonardo da Vinci—</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>will believe</t>
+          <t>Which choice uses punctuation correctly?</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>believe</t>
+          <t>,including Leonardo da Vinci,</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>are believing</t>
+          <t>;including Leonardo da Vinci;</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>believes</t>
+          <t>—including Leonardo da Vinci—</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>:including Leonardo da Vinci:</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>The subject 'a significant number of them' is plural, so the verb should be 'believe' to maintain subject-verb agreement.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>The use of dashes is correct here to set off a nonessential element in the sentence. This provides clarity and conforms to standard written English punctuation rules. Other options incorrectly use commas, semicolons, or colons, which are not appropriate for this structure.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>7f028986-80a6-4790-adf3-adb822742f5f</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Form, Structure, and Sense</t>
-        </is>
-      </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Punctuation</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Despite having conducted numerous controlled experiments, the researchers were unable to determine whether the unexpected results, which had contradicted earlier hypotheses, ______ from measurement error or an unaccounted-for variable.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Despite having conducted numerous controlled experiments, the researchers were unable to determine whether the unexpected results, which had contradicted earlier hypotheses, ______ from measurement error or an unaccounted-for variable.</t>
+          <t>Many historians agree that the Renaissance—a period of cultural rebirth—began in Italy, but they debate how quickly its influence spread to the rest of Europe.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>resulted</t>
+          <t>Many historians agree that the Renaissance—a period of cultural rebirth—began in Italy, but they debate how quickly its influence spread to the rest of Europe.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>—a period of cultural rebirth—</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>resulting</t>
+          <t>Which choice uses punctuation correctly?</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>results</t>
+          <t>—a period of cultural rebirth—</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>resulted</t>
+          <t>(a period of cultural rebirth)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>result</t>
+          <t>: a period of cultural rebirth :</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>, a period of cultural rebirth,</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>The sentence requires the past tense verb 'resulted' to correctly complete the sentence in a grammatically standard way.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>The use of em dashes is correct here as they set off a non-essential element in the sentence, providing additional information without disrupting the main clause.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>37ab8dfb-b1c0-4e75-abd2-2e9c8497366f</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>Standard English Conventions</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Modifiers</t>
-        </is>
-      </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Punctuation</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Walking through the museum, the ancient sculptures fascinated Maya with their intricate designs.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Walking through the museum, the ancient sculptures fascinated Maya with their intricate designs.</t>
+          <t>Although Dr. Lin’s research has been widely cited the underlying methodology—complex and innovative—remains largely misunderstood.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Walking through the museum</t>
+          <t>Although Dr. Lin’s research has been widely cited the underlying methodology—complex and innovative—remains largely misunderstood.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>cited the underlying methodology—complex and innovative—remains</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Walking through the museum,</t>
-        </is>
-      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>In the museum, walking through,</t>
+          <t>cited, the underlying methodology—complex and innovative—remains</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>As she walked through the museum,</t>
+          <t>cited; the underlying methodology—complex and innovative—remains</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>While walking through the museum,</t>
+          <t>cited the underlying methodology—complex and innovative—remains</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>cited: the underlying methodology—complex and innovative—remains</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>The original sentence contains a dangling modifier, as 'Walking through the museum' incorrectly suggests that the ancient sculptures are the ones doing the walking. The correct answer, 'As she walked through the museum,' appropriately links the action with Maya, the intended subject of the modifier.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>A comma is needed after 'cited' to properly separate the dependent clause from the main clause, ensuring the sentence adheres to standard written English.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Standard English Conventions</t>
+          <t>67db20ac-6468-4bd9-ad50-d09ecae491ef</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Modifiers</t>
+          <t>Expression of Ideas</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Transitions</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Eager to present her findings, the research paper was submitted by Dr. Patel before the conference deadline.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Eager to present her findings, the research paper was submitted by Dr. Patel before the conference deadline.</t>
+          <t>Many birds migrate thousands of miles each year to find suitable breeding grounds. However, some species remain in the same area year-round and adapt to changing seasons.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Eager to present her findings,</t>
+          <t>Many birds migrate thousands of miles each year to find suitable breeding grounds. However, some species remain in the same area year-round and adapt to changing seasons.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Which choice best clarifies the intended meaning while following standard written English?</t>
+          <t>However,</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Dr. Patel, eager to present her findings,</t>
+          <t>Which choice best connects the ideas in the text?</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Eager to present, her findings,</t>
+          <t>However,</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Eager to present her findings,</t>
+          <t>Therefore,</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Her findings being eager to present,</t>
+          <t>For example,</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
+          <t>In addition,</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Option A correctly modifies 'Dr. Patel' by placing the descriptive phrase 'eager to present her findings' directly next to the noun it is intended to describe, clarifying the intended meaning and improving grammatical correctness.</t>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>The transition 'However,' correctly indicates a contrast between the migration of many bird species and the stationary behavior of others, which is the logical relationship intended by the passage.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Standard English Conventions</t>
+          <t>9710160f-bae6-409c-8ac8-c7f07ba1caa9</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Modifiers</t>
+          <t>Expression of Ideas</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Transitions</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>While analyzing the ancient manuscript, the historians found it difficult to decipher the original text because of the faded ink.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>While analyzing the ancient manuscript, the historians found it difficult to decipher the original text because of the faded ink.</t>
+          <t>The artist experimented with vibrant colors to evoke emotion in her paintings. [Transition], she also paid close attention to the use of light and shadow to create depth.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>While analyzing the ancient manuscript,</t>
+          <t>The artist experimented with vibrant colors to evoke emotion in her paintings. [Transition], she also paid close attention to the use of light and shadow to create depth.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>[Transition]</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>While analyzing the ancient manuscript,</t>
+          <t>Which choice completes the text with the most logical transition?</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>While the ancient manuscript was analyzing,</t>
+          <t>However,</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>While the ancient manuscript was being analyzed by,</t>
+          <t>In addition,</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>While the ancient manuscript analyzed,</t>
+          <t>Therefore,</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Consequently,</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Option A correctly places the modifier 'While analyzing the ancient manuscript,' to indicate that 'the historians' were performing the action, avoiding a dangling modifier error present in the other options.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>The correct transition should indicate that the second idea is an additional aspect of the artist's technique. 'In addition,' effectively conveys that the artist's attention to light and shadow complements her use of vibrant colors, rather than contrasting with or resulting from it.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Standard English Conventions</t>
+          <t>7c8d5586-7703-433c-8a44-bc10d9b37c55</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Punctuation</t>
+          <t>Expression of Ideas</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Transitions</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Dr. Ramirez studied the fossils carefully but she could not determine the species.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Dr. Ramirez studied the fossils carefully but she could not determine the species.</t>
+          <t>Many ancient civilizations developed writing systems to record agricultural yields. Nevertheless, some communities relied exclusively on oral traditions to preserve their histories.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>but she could not determine the species</t>
+          <t>Many ancient civilizations developed writing systems to record agricultural yields. Nevertheless, some communities relied exclusively on oral traditions to preserve their histories.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>Nevertheless,</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>but, she could not determine the species.</t>
+          <t>Which choice best connects the ideas in the text?</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>: but she could not determine the species.</t>
+          <t>For example,</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>, but she could not determine the species.</t>
+          <t>Nevertheless,</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>; but she could not determine the species.</t>
+          <t>As a result,</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Furthermore,</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>In standard written English, a comma is needed before a conjunction like 'but' when it is used to join two independent clauses. Therefore, option A correctly uses a comma to separate the clauses.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>The passage presents a contrast between two different approaches to preserving historical records: writing systems and oral traditions. 'Nevertheless' appropriately signals this contrast.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Standard English Conventions</t>
+          <t>980d35f3-d4bb-4c9f-8a57-fb77be80f8a6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Punctuation</t>
+          <t>Expression of Ideas</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Organization</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>In her groundbreaking research, Dr. Morales demonstrated that the new treatment was not only effective in reducing symptoms[editable_portion] it also improved patients' overall quality of life.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>In her groundbreaking research, Dr. Morales demonstrated that the new treatment was not only effective in reducing symptoms[editable_portion] it also improved patients' overall quality of life.</t>
+          <t>Honeybees play a crucial role in pollinating many crops. For example, without honeybees, the production of apples, almonds, and blueberries would decrease significantly. Many farmers rely on these insects to help their plants grow healthy fruits.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>;</t>
+          <t>Honeybees play a crucial role in pollinating many crops. For example, without honeybees, the production of apples, almonds, and blueberries would decrease significantly. Many farmers rely on these insects to help their plants grow healthy fruits.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>For example, without honeybees, the production of apples, almonds, and blueberries would decrease significantly.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>;</t>
+          <t>Which choice most logically completes the text?</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>and</t>
+          <t>As a result, the production of apples, almonds, and blueberries would remain the same without honeybees.</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>,</t>
+          <t>For example, without honeybees, the production of apples, almonds, and blueberries would decrease significantly.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>In contrast, without honeybees, the production of apples, almonds, and blueberries would increase significantly.</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Therefore, the production of apples, almonds, and blueberries would decrease significantly without honeybees.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>The semicolon is the correct choice because it properly separates two independent clauses without the need for a conjunction, in accordance with standard English conventions.</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Option A logically follows the introduction of honeybees' role by providing an example of their impact on crop production, which enhances the coherence and flow of the passage.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Standard English Conventions</t>
+          <t>5ce29f7f-e913-4a51-8166-0211587378d5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Punctuation</t>
+          <t>Expression of Ideas</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Organization</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>The physicist’s theory—which was initially dismissed by her peers—eventually gained recognition; it explained phenomena that, until then, had been misunderstood.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>The physicist’s theory—which was initially dismissed by her peers—eventually gained recognition; it explained phenomena that, until then, had been misunderstood.</t>
+          <t>Researchers observed that the migratory patterns of monarch butterflies have changed over the past decade. However, studies focusing on pesticide use have also revealed significant impacts on butterfly populations. This shift is believed to be linked to fluctuations in regional temperatures, suggesting multiple factors may be involved.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>—which was initially dismissed by her peers—</t>
+          <t>Researchers observed that the migratory patterns of monarch butterflies have changed over the past decade. However, studies focusing on pesticide use have also revealed significant impacts on butterfly populations. This shift is believed to be linked to fluctuations in regional temperatures, suggesting multiple factors may be involved.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Which choice completes the text so that it conforms to the conventions of Standard English?</t>
+          <t>However, studies focusing on pesticide use have also revealed significant impacts on butterfly populations.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>, which was initially dismissed by her peers,</t>
+          <t>Which choice best improves the organization of the passage?</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>--which was initially dismissed by her peers--</t>
+          <t>Move the sentence to the end of the paragraph.</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>which was initially dismissed by her peers,</t>
+          <t>Delete the sentence entirely.</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>—which was initially dismissed by her peers—</t>
+          <t>Move the sentence to the beginning of the paragraph.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Leave the sentence where it is.</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>The use of the em dash (—) correctly sets off the nonrestrictive clause 'which was initially dismissed by her peers' from the main clause. This choice maintains the intended emphasis and separation of ideas within the sentence structure.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Moving the sentence to the end of the paragraph enhances the logical progression by first discussing the observed changes and then suggesting multiple factors, including pesticide use, that may be responsible.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>5556251a-07a1-4726-8389-adf63bc9a0c9</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Transitions</t>
-        </is>
-      </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Organization</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Birds are able to travel thousands of miles during migration. However, some smaller species remain in the same area year-round.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Birds are able to travel thousands of miles during migration. However, some smaller species remain in the same area year-round.</t>
+          <t>The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. In addition, these pieces are now considered pivotal by art historians. She began experimenting with color theory during this period, a technique that became central to her mature paintings.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>However,</t>
+          <t>The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. In addition, these pieces are now considered pivotal by art historians. She began experimenting with color theory during this period, a technique that became central to her mature paintings.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Which choice best connects the ideas in the text?</t>
+          <t>In addition, these pieces are now considered pivotal by art historians.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Additionally,</t>
+          <t>Which choice best improves the organization of the passage?</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>However,</t>
+          <t>She began experimenting with color theory during this period, a technique that became central to her mature paintings. The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. In addition, these pieces are now considered pivotal by art historians.</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>For example,</t>
+          <t>In addition, these pieces are now considered pivotal by art historians. The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. She began experimenting with color theory during this period, a technique that became central to her mature paintings.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Therefore,</t>
+          <t>The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. She began experimenting with color theory during this period, a technique that became central to her mature paintings. In addition, these pieces are now considered pivotal by art historians.</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>The artist’s early works, though often overlooked by critics at the time, reveal the foundations of her later style. In addition, these pieces are now considered pivotal by art historians. She began experimenting with color theory during this period, a technique that became central to her mature paintings.</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>The sentence contrasts the ability of birds to migrate long distances with the fact that some smaller species do not migrate, making 'However,' the most logical transition.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Option A maintains a logical progression by first discussing the early works' foundational role and experimentation with color theory, followed by the recognition of their importance, keeping the ideas coherently connected.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>8fdeaf97-ecd8-4f2b-8945-097574cc3965</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Transitions</t>
-        </is>
-      </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Concision and Precision</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Marie Curie’s groundbreaking research on radioactivity earned her two Nobel Prizes. [However/For example/As a result/In addition], she often faced significant obstacles due to her status as a woman in science.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Marie Curie’s groundbreaking research on radioactivity earned her two Nobel Prizes. [However/For example/As a result/In addition], she often faced significant obstacles due to her status as a woman in science.</t>
+          <t>The scientist conducted an experiment that was designed in order to test whether plants grow faster when exposed to more sunlight.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[However/For example/As a result/In addition]</t>
+          <t>The scientist conducted an experiment that was designed in order to test whether plants grow faster when exposed to more sunlight.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Which choice best connects the ideas in the text?</t>
+          <t>conducted an experiment that was designed in order to</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>For example</t>
+          <t>Which choice is the clearest and most concise?</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>In addition</t>
+          <t>conducted an experiment with the purpose of</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>However</t>
+          <t>conducted a designed experiment for the purpose of</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>As a result</t>
+          <t>conducted an experiment that was designed in order to</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>conducted an experiment to</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>The passage presents a contrast between Marie Curie's achievements and the challenges she faced. 'However' appropriately highlights this contrast, while the other options suggest relationships that do not logically fit the context.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Option A is the most concise and eliminates unnecessary words found in the other options.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>574b0968-b11e-461c-89ea-54f4075a2f12</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Transitions</t>
-        </is>
-      </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Concision and Precision</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Researchers initially hypothesized that the observed decline in bee populations was due to pesticide exposure. Nevertheless, subsequent studies revealed that habitat loss played a more significant role.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Researchers initially hypothesized that the observed decline in bee populations was due to pesticide exposure. Nevertheless, subsequent studies revealed that habitat loss played a more significant role.</t>
+          <t>In her analysis of the novel, Dr. Chen argues that the protagonist’s journey, which is a trip that spans several continents, is essential to the book’s theme of self-discovery.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Nevertheless</t>
+          <t>In her analysis of the novel, Dr. Chen argues that the protagonist’s journey, which is a trip that spans several continents, is essential to the book’s theme of self-discovery.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Which choice best connects the ideas in the text?</t>
+          <t>which is a trip that spans several continents</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>As a result,</t>
+          <t>Which choice is the clearest and most concise?</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>For example,</t>
+          <t>spanning several continents</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>In contrast,</t>
+          <t>going through various continents</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Moreover,</t>
+          <t>that spans across a number of continents</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>which is a trip that spans several continents</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>The transition 'In contrast,' correctly highlights the shift from the initial hypothesis about pesticide exposure to the subsequent finding about habitat loss, indicating a contrast between the two findings.</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Option A is the most concise and clear way to express the idea without unnecessary words or redundancy. It effectively conveys the scope of the journey in a direct manner.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>0f84e8b8-010b-457a-b7d7-678dd5854d31</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Concision and Precision</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Bees play a vital role in pollinating plants. However, their populations are declining due to factors such as pesticide use and habitat loss. For example, wildflower meadows that once supported many bees have been replaced by farmland. This makes the protection of bee habitats especially important.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Bees play a vital role in pollinating plants. However, their populations are declining due to factors such as pesticide use and habitat loss. For example, wildflower meadows that once supported many bees have been replaced by farmland. This makes the protection of bee habitats especially important.</t>
+          <t>Due to the fact that the experiment yielded results that were unexpected and not in accordance with the hypothesis, the researchers decided to conduct additional trials to clarify their findings.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>For example, wildflower meadows that once supported many bees have been replaced by farmland.</t>
+          <t>Due to the fact that the experiment yielded results that were unexpected and not in accordance with the hypothesis, the researchers decided to conduct additional trials to clarify their findings.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Which choice most logically completes the text?</t>
+          <t>Due to the fact that</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>For example, wildflower meadows that once supported many bees have been replaced by farmland.</t>
+          <t>Which choice is the clearest and most concise?</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>However, wildflower meadows have been replaced by farmland, affecting bees.</t>
+          <t>Because</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Moreover, wildflower meadows have been replaced by farmland, which supports bees.</t>
+          <t>In light of the fact that</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>In contrast, wildflower meadows are replaced by farmland that bees avoid.</t>
+          <t>As a result of</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
+          <t>Due to the fact that</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>Option A maintains the logical progression of ideas by providing a specific example of habitat loss, which supports the statement about the decline of bee populations due to habitat loss.</t>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Option A is the clearest and most concise way to express the cause-effect relationship in the sentence. The other options are unnecessarily wordy.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>17a1bb12-6d60-4c2d-b89f-9679b55b2778</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Rhetorical Synthesis</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>The telescope was invented in the early 17th century, revolutionizing astronomy. Galileo Galilei, for example, used it to observe Jupiter’s moons. He also recorded detailed drawings of the lunar surface, revealing features such as mountains and craters. These discoveries challenged the prevailing view that all celestial bodies revolved around Earth.</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>The telescope was invented in the early 17th century, revolutionizing astronomy. Galileo Galilei, for example, used it to observe Jupiter’s moons. He also recorded detailed drawings of the lunar surface, revealing features such as mountains and craters. These discoveries challenged the prevailing view that all celestial bodies revolved around Earth.</t>
+          <t>Many scientists have studied the migration patterns of monarch butterflies; to highlight recent changes, the writer wants to introduce a sentence that summarizes the main findings of a 2022 study showing that rising temperatures have shifted both the timing and routes of monarch migrations. Their research suggests that changing temperatures are causing monarchs to start their journeys earlier each year.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>He also recorded detailed drawings of the lunar surface, revealing features such as mountains and craters.</t>
+          <t>Many scientists have studied the migration patterns of monarch butterflies; to highlight recent changes, the writer wants to introduce a sentence that summarizes the main findings of a 2022 study showing that rising temperatures have shifted both the timing and routes of monarch migrations. Their research suggests that changing temperatures are causing monarchs to start their journeys earlier each year.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Which choice best improves the organization of the passage?</t>
+          <t>a sentence that summarizes the main findings of a 2022 study showing that rising temperatures have shifted both the timing and routes of monarch migrations.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>He recorded detailed observations of the lunar surface, which included mountains and craters.</t>
+          <t>Which choice most effectively uses relevant information from the notes to accomplish the writer's goal of summarizing the main findings of a 2022 study?</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Revealing features such as mountains and craters, he also recorded detailed drawings of the lunar surface.</t>
+          <t>A 2022 study highlighted the routes of monarch migrations without focusing on temperature changes.</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>He also recorded detailed drawings of the lunar surface, revealing features such as mountains and craters.</t>
+          <t>A 2022 study suggested that monarch butterflies are migrating differently, but did not mention temperatures.</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Details such as mountains and craters were revealed in his recorded drawings of the lunar surface.</t>
+          <t>A 2022 study discovered various factors affecting monarch migrations, with temperature being a minor influence.</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A 2022 study found that rising temperatures are prompting monarch butterflies to migrate earlier and along different routes.</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Option A maintains the chronological and logical flow of the passage, which discusses Galileo's use of the telescope for astronomical observations. It effectively follows the previous sentence about his observations of Jupiter’s moons, without unnecessary disruption or rephrasing that could obstruct the logical progression.</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Option A directly summarizes the main findings of the 2022 study, clearly linking rising temperatures to changes in the timing and routes of monarch migrations, aligning with the writer's goal.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>7602737e-6167-499d-8e8b-33c06ec38b2f</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Rhetorical Synthesis</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>The telescope’s ability to gather faint light from distant galaxies has revolutionized our understanding of the universe. However, its discoveries would not have been possible without the development of advanced imaging techniques, which allow astronomers to capture clearer, more detailed images. [Where should the previous sentence be placed for the best logical flow?] Originally, astronomers relied on less sensitive instruments that limited their observations.</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>The telescope’s ability to gather faint light from distant galaxies has revolutionized our understanding of the universe. However, its discoveries would not have been possible without the development of advanced imaging techniques, which allow astronomers to capture clearer, more detailed images. [Where should the previous sentence be placed for the best logical flow?] Originally, astronomers relied on less sensitive instruments that limited their observations.</t>
+          <t>Researchers examined several urban areas and found that city parks not only provide recreational spaces but also help reduce air pollution, a finding that has important implications for public health policy.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[Where should the previous sentence be placed for the best logical flow?]</t>
+          <t>Researchers examined several urban areas and found that city parks not only provide recreational spaces but also help reduce air pollution, a finding that has important implications for public health policy.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Where should the previous sentence be placed for the best logical flow?</t>
+          <t>a finding that has important implications for public health policy</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>At the end of the passage.</t>
+          <t>Which choice most effectively emphasizes the significance of the researchers' findings for broader societal concerns?</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Before the first sentence.</t>
+          <t>a finding that may change how people view city parks</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>After the first sentence.</t>
+          <t>a finding that suggests potential improvements in urban planning</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>After the second sentence.</t>
+          <t>a finding that has important implications for public health policy</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>a finding that indicates a need for further research</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Placing the sentence after the second sentence provides a logical progression from the limitations of earlier instruments to the advancements that made new discoveries possible, improving the overall coherence of the passage.</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Option A directly relates the findings to public health policy, emphasizing their broader societal implications, which aligns with the context of the passage.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>f1b2843e-77df-4c01-a58f-fd39f29dcad6</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>Expression of Ideas</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Concision and Precision</t>
-        </is>
-      </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Rhetorical Synthesis</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Because of the fact that photosynthesis allows plants to convert sunlight into energy, it plays a crucial role in sustaining life on Earth.</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Because of the fact that photosynthesis allows plants to convert sunlight into energy, it plays a crucial role in sustaining life on Earth.</t>
+          <t>Recent archaeological discoveries in the Andes have revealed evidence of advanced agricultural terraces, intricate irrigation systems, and domesticated crops, ________________, highlighting the resourcefulness of ancient civilizations in adapting to challenging environmental conditions.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Because of the fact that</t>
+          <t>Recent archaeological discoveries in the Andes have revealed evidence of advanced agricultural terraces, intricate irrigation systems, and domesticated crops, ________________, highlighting the resourcefulness of ancient civilizations in adapting to challenging environmental conditions.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Which choice is the clearest and most concise?</t>
+          <t>which together provide a comprehensive view of how these societies managed scarce water resources</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>As a result of the fact that</t>
+          <t>Which choice most effectively synthesizes the information about ancient civilizations' resourcefulness in the Andes?</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Because</t>
+          <t>which were not as advanced as previously thought</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Due to the fact that</t>
+          <t>which together provide a comprehensive view of how these societies managed scarce water resources</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>For the reason that</t>
+          <t>which resulted in the downfall of neighboring civilizations</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
+          <t>which contrast with the simpler societies that did not adapt as well</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>Option A 'Because' is the clearest and most concise way to convey the causal relationship in the sentence. The other options are wordier and less direct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Expression of Ideas</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Concision and Precision</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Although the painting was created in the twentieth century, it nevertheless continues, even today, to attract the attention of art critics around the world.</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Although the painting was created in the twentieth century, it nevertheless continues, even today, to attract the attention of art critics around the world.</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>nevertheless continues, even today, to attract the attention of</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Which choice is the clearest and most concise?</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>still keeps attracting</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>remains continuing to attract</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>continues to attract</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>nevertheless continues, even today, to attract</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Option A is the clearest and most concise choice, removing unnecessary words while retaining the original meaning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Expression of Ideas</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Concision and Precision</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Although the experiment was conducted in a laboratory setting that was controlled and free from external variables, unintended factors may have influenced the outcomes in ways that were not predicted by the researchers.</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Although the experiment was conducted in a laboratory setting that was controlled and free from external variables, unintended factors may have influenced the outcomes in ways that were not predicted by the researchers.</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>in ways that were not predicted by the researchers</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Which choice most effectively conveys the idea?</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>unpredictably</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>in a manner that was unforeseen by them</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>unexpectedly</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>in ways that were not predicted by the researchers</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>Option A, 'unexpectedly', is the most concise and precise way to convey the idea that the outcomes were not predicted by the researchers, avoiding redundancy and unnecessary wordiness present in the other options.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Expression of Ideas</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Rhetorical Synthesis</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Fossil evidence indicates that some ancient whales had small hind limbs, a fact that reveals how these marine mammals evolved from land-dwelling ancestors. To best emphasize the importance of this discovery, which choice most effectively highlights the significance of the hind limb fossils?</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Fossil evidence indicates that some ancient whales had small hind limbs, a fact that reveals how these marine mammals evolved from land-dwelling ancestors. To best emphasize the importance of this discovery, which choice most effectively highlights the significance of the hind limb fossils?</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>To best emphasize the importance of this discovery, which choice most effectively highlights the significance of the hind limb fossils?</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>To best emphasize the importance of this discovery, which choice most effectively highlights the significance of the hind limb fossils?</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>The presence of hind limbs in ancient whales underscores their evolution from terrestrial ancestors.</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Hind limb fossils are just one piece of evidence in the study of whale evolution.</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Whale fossils are often found with other marine life fossils, providing context.</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Some ancient whales had hind limbs, which is a curious fact about their anatomy.</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Option A most effectively highlights the significance of the hind limb fossils by directly connecting them to the evolution of whales from land-dwelling ancestors, thus emphasizing the importance of the discovery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Expression of Ideas</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Rhetorical Synthesis</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Recently, researchers have explored how urban green spaces affect residents’ mental health; however, studies differ in their findings, with some showing significant benefits and others reporting minimal effects.</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Recently, researchers have explored how urban green spaces affect residents’ mental health; however, studies differ in their findings, with some showing significant benefits and others reporting minimal effects.</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>with some showing significant benefits and others reporting minimal effects</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Which choice best supports the writer's purpose of conveying the varying impact of urban green spaces on mental health?</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>with some showing significant benefits and others reporting minimal effects</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>with studies showing mixed effects but generally positive trends</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>with all studies agreeing on the benefits</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>with some studies reporting no benefits at all</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>Option A most effectively conveys the idea of differing study results, which aligns with the writer's purpose of highlighting the variability in research findings about urban green spaces and mental health.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Expression of Ideas</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Rhetorical Synthesis</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Recent archaeological discoveries in the Mediterranean region have revealed unexpected trade connections between ancient civilizations; [best way to introduce the significance of these findings], these artifacts suggest that cross-cultural exchange occurred much earlier than previously believed.</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Recent archaeological discoveries in the Mediterranean region have revealed unexpected trade connections between ancient civilizations; [best way to introduce the significance of these findings], these artifacts suggest that cross-cultural exchange occurred much earlier than previously believed.</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>[best way to introduce the significance of these findings]</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Which choice most effectively introduces the significance of the findings in the passage?</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>these findings have been anticipated by historians,</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>these findings are similar to previous discoveries,</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>these findings are interesting to archaeologists,</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>these findings redefine our understanding of early trade networks,</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>Option A is the most relevant and effective because it emphasizes the significant impact of the discoveries on our understanding of early trade networks, aligning with the context of unexpected trade connections. The other options are less focused on the significance or are factually possible but less relevant.</t>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Option A accurately completes the sentence by highlighting the resourcefulness of ancient civilizations in managing scarce water resources, which aligns with the context of the passage. The other options introduce unrelated or inaccurate information.</t>
         </is>
       </c>
     </row>

</xml_diff>